<commit_message>
Add Lesson 8 data cleaning and Lesson 9 chart generation
</commit_message>
<xml_diff>
--- a/master_all_folder_sales.xlsx
+++ b/master_all_folder_sales.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -499,94 +499,117 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Department</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D5" t="n">
+        <v>15000</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>employees.xlsx</t>
+          <t>calculated_sales.xlsx</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>U Aung</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>4500000</v>
+        <v>2000</v>
+      </c>
+      <c r="D6" t="n">
+        <v>10000</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>employees.xlsx</t>
+          <t>calculated_sales.xlsx</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Daw Hla</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Marketing</t>
-        </is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>12</v>
       </c>
       <c r="C7" t="n">
-        <v>1800000</v>
+        <v>500</v>
+      </c>
+      <c r="D7" t="n">
+        <v>6000</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>employees.xlsx</t>
+          <t>calculated_sales.xlsx</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Ko Tun</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>6000000</v>
+          <t>Department</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
           <t>employees.xlsx</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Ma Su</t>
+          <t>U Aung</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -595,45 +618,48 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2500000</v>
+        <v>4500000</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
           <t>employees.xlsx</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Daw Hla</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Department</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1800000</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>employees_evaluated.xlsx</t>
+          <t>employees.xlsx</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>U Aung</t>
+          <t>Ko Tun</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -642,58 +668,80 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>4500000</v>
+        <v>6000000</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>employees_evaluated.xlsx</t>
+          <t>employees.xlsx</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Daw Hla</t>
+          <t>Ma Su</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1800000</v>
+        <v>2500000</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>employees_evaluated.xlsx</t>
+          <t>employees.xlsx</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Ko Tun</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>6000000</v>
+          <t>Department</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
           <t>employees_evaluated.xlsx</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Ma Su</t>
+          <t>U Aung</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -702,62 +750,91 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2500000</v>
+        <v>4500000</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
           <t>employees_evaluated.xlsx</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Orange</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>200</v>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>february_sales.xlsx</t>
+          <t>Daw Hla</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>employees_evaluated.xlsx</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Mango</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>250</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>february_sales.xlsx</t>
+          <t>Ko Tun</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>employees_evaluated.xlsx</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Apple</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>10</v>
+          <t>Ma Su</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
       </c>
       <c r="C17" t="n">
-        <v>1500</v>
-      </c>
-      <c r="D17" t="n">
-        <v>15000</v>
+        <v>2500000</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>filtered_sorted_sales.xlsx</t>
+          <t>employees_evaluated.xlsx</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
         </is>
       </c>
     </row>
@@ -768,38 +845,36 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>5</v>
-      </c>
-      <c r="C18" t="n">
-        <v>2000</v>
-      </c>
-      <c r="D18" t="n">
-        <v>10000</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>filtered_sorted_sales.xlsx</t>
+        <v>200</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>february_sales.xlsx</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Banana</t>
+          <t>Mango</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>12</v>
-      </c>
-      <c r="C19" t="n">
-        <v>500</v>
-      </c>
-      <c r="D19" t="n">
-        <v>6000</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>filtered_sorted_sales.xlsx</t>
+        <v>250</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>february_sales.xlsx</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
         </is>
       </c>
     </row>
@@ -815,9 +890,17 @@
       <c r="C20" t="n">
         <v>1500</v>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>first_automation.xlsx</t>
+      <c r="D20" t="n">
+        <v>15000</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>filtered_sorted_sales.xlsx</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
         </is>
       </c>
     </row>
@@ -833,9 +916,17 @@
       <c r="C21" t="n">
         <v>2000</v>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>first_automation.xlsx</t>
+      <c r="D21" t="n">
+        <v>10000</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>filtered_sorted_sales.xlsx</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
         </is>
       </c>
     </row>
@@ -851,9 +942,17 @@
       <c r="C22" t="n">
         <v>500</v>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>first_automation.xlsx</t>
+      <c r="D22" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>filtered_sorted_sales.xlsx</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
         </is>
       </c>
     </row>
@@ -864,174 +963,855 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>100</v>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>january_sales.xlsx</t>
+        <v>10</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>first_automation.xlsx</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>5</v>
+      </c>
+      <c r="C24" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>first_automation.xlsx</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>Banana</t>
         </is>
       </c>
-      <c r="B24" t="n">
-        <v>150</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>january_sales.xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
+      <c r="B25" t="n">
+        <v>12</v>
+      </c>
+      <c r="C25" t="n">
+        <v>500</v>
+      </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>merged_master_report.xlsx</t>
+          <t>first_automation.xlsx</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Ko Tun</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>6000000</v>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>merged_master_report.xlsx</t>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>100</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>january_sales.xlsx</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>U Aung</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>4500000</v>
-      </c>
-      <c r="D27" t="inlineStr">
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>150</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>january_sales.xlsx</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="D28" t="inlineStr">
         <is>
           <t>merged_master_report.xlsx</t>
         </is>
       </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Ma Su</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>2500000</v>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>merged_master_report.xlsx</t>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Daw Hla</t>
+          <t>Ko Tun</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1800000</v>
+        <v>6000000</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
           <t>merged_master_report.xlsx</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Apple</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>10</v>
+          <t>U Aung</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
       </c>
       <c r="C30" t="n">
-        <v>1500</v>
-      </c>
-      <c r="D30" t="n">
-        <v>15000</v>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>styled_sales.xlsx</t>
+        <v>4500000</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>merged_master_report.xlsx</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Orange</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>5</v>
+          <t>Ma Su</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
       </c>
       <c r="C31" t="n">
-        <v>2000</v>
-      </c>
-      <c r="D31" t="n">
-        <v>10000</v>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>styled_sales.xlsx</t>
+        <v>2500000</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>merged_master_report.xlsx</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>Daw Hla</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>merged_master_report.xlsx</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>10</v>
+      </c>
+      <c r="C33" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D33" t="n">
+        <v>15000</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>styled_sales.xlsx</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>5</v>
+      </c>
+      <c r="C34" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D34" t="n">
+        <v>10000</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>styled_sales.xlsx</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>Banana</t>
         </is>
       </c>
-      <c r="B32" t="n">
+      <c r="B35" t="n">
         <v>12</v>
       </c>
-      <c r="C32" t="n">
+      <c r="C35" t="n">
         <v>500</v>
       </c>
-      <c r="D32" t="n">
+      <c r="D35" t="n">
         <v>6000</v>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>styled_sales.xlsx</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>cleaned_sales_data.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Department</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>employees.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>U Aung</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>4500000</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>employees.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Daw Hla</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>employees.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Ko Tun</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>employees.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Ma Su</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>employees.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Department</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>employees_evaluated.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>U Aung</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>4500000</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>employees_evaluated.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Daw Hla</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>employees_evaluated.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Ko Tun</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>employees_evaluated.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Ma Su</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>employees_evaluated.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>200</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>february_sales.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Mango</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>250</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>february_sales.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>10</v>
+      </c>
+      <c r="C48" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D48" t="n">
+        <v>15000</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>filtered_sorted_sales.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>5</v>
+      </c>
+      <c r="C49" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D49" t="n">
+        <v>10000</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>filtered_sorted_sales.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>12</v>
+      </c>
+      <c r="C50" t="n">
+        <v>500</v>
+      </c>
+      <c r="D50" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>filtered_sorted_sales.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>10</v>
+      </c>
+      <c r="C51" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>first_automation.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>5</v>
+      </c>
+      <c r="C52" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>first_automation.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>12</v>
+      </c>
+      <c r="C53" t="n">
+        <v>500</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>first_automation.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>100</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>january_sales.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>150</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>january_sales.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>merged_master_report.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Ko Tun</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>merged_master_report.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>U Aung</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>4500000</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>merged_master_report.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Ma Su</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>merged_master_report.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Daw Hla</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>merged_master_report.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>10</v>
+      </c>
+      <c r="C61" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D61" t="n">
+        <v>15000</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>polars_filtered.sales.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>10</v>
+      </c>
+      <c r="C62" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D62" t="n">
+        <v>15000</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>styled_sales.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>5</v>
+      </c>
+      <c r="C63" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D63" t="n">
+        <v>10000</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>styled_sales.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Banana</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>12</v>
+      </c>
+      <c r="C64" t="n">
+        <v>500</v>
+      </c>
+      <c r="D64" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E64" t="inlineStr">
         <is>
           <t>styled_sales.xlsx</t>
         </is>

</xml_diff>